<commit_message>
site build 2026-10-08 21:14
</commit_message>
<xml_diff>
--- a/models/sovereigns/Egypt_Sovereign_Model.xlsx
+++ b/models/sovereigns/Egypt_Sovereign_Model.xlsx
@@ -647,12 +647,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sep-26 (overnight deposit rate; lending rate 20.00)</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CBE Monetary Policy Committee</t>
+          <t>Central Bank of Egypt MPC decision (overnight deposit rate; lending rate 20.00%)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Aug-26 (nationwide headline; urban 14.5)</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CAPMAS August 2026 CPI Bulletin</t>
+          <t>CAPMAS (nationwide headline; urban 14.5%)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -739,11 +739,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -778,7 +774,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026 (Q2-26)</t>
+          <t>Q2-26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>General budget sector debt</t>
+          <t>Budget-sector perimeter only; source mixes MoF and IIF figures (96.4% in FY23/24)</t>
         </is>
       </c>
     </row>
@@ -804,7 +800,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -813,12 +809,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FY2024/25 (audited; FY2025/26 target 4.0)</t>
+          <t>FY25/26 (budget)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Finance of Egypt</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -849,7 +845,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (overall balance)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -857,11 +853,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -961,11 +953,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -996,11 +984,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1018,7 +1002,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1028,12 +1012,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
+          <t>IMF International Liquidity, gross incl. gold (ex-gold 36.42, gold 17.139)</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1037,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>end-Sep-26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1068,7 +1052,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CBE net international reserves, record high; treatment of swaps and foreign bank liabilities not confirmed (open item)</t>
+          <t>CBE net international reserves; definition not reconciled with IMF gross series, not comparable</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1072,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sep-26 (reported as over 7.5 months of merchandise imports)</t>
+          <t>end-Sep-26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Central Bank of Egypt</t>
+          <t>Central Bank of Egypt (reported as over 7.5 months)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1183,11 +1167,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1297,7 +1277,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>01-Nov-24</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1299,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>10-Oct-25</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1321,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>18-Mar-24</t>
         </is>
       </c>
     </row>
@@ -1358,11 +1338,6 @@
       </c>
       <c r="C33" t="n">
         <v>8</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Mar-24 (expanded to $8B)</t>
-        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1381,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1415,10 +1390,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>FY25/26</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>FY25/26E</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Q2-26</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1431,11 +1416,19 @@
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
+        <v>429.645</v>
+      </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1444,11 +1437,19 @@
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="n">
+        <v>4.2</v>
+      </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1461,7 +1462,9 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1470,11 +1473,19 @@
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v>-4.2</v>
+      </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1483,11 +1494,19 @@
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="n">
+        <v>-12.1</v>
+      </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1508,9 +1527,13 @@
       <c r="F7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Ministry of Finance, Sep-26 (fiscal years: 2025 = FY2024/25 audited, 2026E = FY2025/26 target)</t>
+      <c r="G7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ministry of Finance of Egypt, Sep-26 (FY24/25 outturn, FY25/26 budget)</t>
         </is>
       </c>
     </row>
@@ -1529,9 +1552,13 @@
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Ministry of Finance / IIF, Jun-26 (general budget sector debt)</t>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ministry of Finance / IIF, Jun-26 (budget-sector perimeter)</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1573,9 @@
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1559,7 +1588,9 @@
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1572,7 +1603,9 @@
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1585,7 +1618,9 @@
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
site build 2026-10-15 08:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Egypt_Sovereign_Model.xlsx
+++ b/models/sovereigns/Egypt_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/egypt.json</t>
+          <t>built 15-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/egypt.json</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Central Bank of Egypt MPC decision (overnight deposit rate; lending rate 20.00%)</t>
+          <t>CBE MPC, overnight deposit rate, via BNOK24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -695,17 +695,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CAPMAS (nationwide headline; urban 14.5%)</t>
+          <t>CAPMAS via Arab Finance (nationwide headline)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10-Sep-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -779,7 +779,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ministry of Finance / IIF</t>
+          <t>MoF / IIF</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>budget sector only; source mixes MoF and IIF figures</t>
+          <t>budget-sector debt</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4</v>
+        <v>4.9</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -809,17 +809,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FY25/26 (budgeted; FY24/25 outturn 3.5)</t>
+          <t>FY25/26</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ministry of Finance of Egypt</t>
+          <t>S&amp;P via Arab News (MoF budgeted 4.0%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>11-Oct-26</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -845,12 +845,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO (overall balance)</t>
+          <t>IMF WEO (overall deficit)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -888,17 +888,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jun-26 (lower bound, reported as more than 50%)</t>
+          <t>FY25/26</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ministry of Finance / IIF</t>
+          <t>S&amp;P via Arab News (MoF/IIF: more than 50%, lower bound)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>11-Oct-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -946,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross incl. gold (ex-gold 36.42; gold 17.139)</t>
+          <t>gross incl. gold (IMF International Liquidity)</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CBE net international reserves, as reported; net forward/swap treatment not confirmed and not reconcilable with IMF gross figure</t>
+          <t>CBE-reported net international reserves; definition unverified and exceeds IMF gross, not comparable</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Central Bank of Egypt (reported as over 7.5 months)</t>
+          <t>Central Bank of Egypt (over 7.5 months)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>429.645</v>
+        <v>429.6</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>01-Nov-24</t>
+          <t>Oct-26</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10-Oct-25</t>
+          <t>11-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>18-Mar-24</t>
+          <t>Apr-26</t>
         </is>
       </c>
     </row>
@@ -1332,17 +1332,14 @@
           <t>EFF (with RSF)</t>
         </is>
       </c>
-      <c r="C33" t="n">
-        <v>8</v>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Seventh Review completed 31-Jul-26, $1.8B approved ($1.5B EFF, $272M RSF)</t>
+          <t>31-Jul-26 (Seventh Review completed, $1.8B)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 (Eighth and final review)</t>
+          <t>15-Dec-26 (Eighth and final review; no primary source)</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1415,7 @@
       </c>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n">
-        <v>429.645</v>
+        <v>429.6</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -1427,7 +1424,7 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1445,7 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1481,7 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1502,7 @@
       <c r="H6" s="2" t="n"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 15-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-23 08:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Egypt_Sovereign_Model.xlsx
+++ b/models/sovereigns/Egypt_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 15-Oct-26</t>
+          <t>as of 23-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/egypt.json</t>
+          <t>built 23-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/egypt.json</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CBE MPC, overnight deposit rate, via BNOK24</t>
+          <t>CBE overnight deposit rate, MPC decision via BNOK24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CAPMAS via Arab Finance (nationwide headline)</t>
+          <t>CAPMAS via Arab Finance</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>10-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>79.7</v>
+        <v>81.8</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -774,22 +774,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Q2-26</t>
+          <t>Jun-26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MoF / IIF</t>
+          <t>Moody's via Daba Finance</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>budget-sector debt</t>
+          <t>public debt as reported by Moody's; MoF/IIF budget-sector figure is 79.7% at Q2-26 on a different perimeter</t>
         </is>
       </c>
     </row>
@@ -814,12 +814,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>S&amp;P via Arab News (MoF budgeted 4.0%)</t>
+          <t>Moody's and S&amp;P via press</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -893,12 +893,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>S&amp;P via Arab News (MoF/IIF: more than 50%, lower bound)</t>
+          <t>Moody's via Daba Finance (S&amp;P puts it at 67%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>11-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -941,7 +941,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO via repo record</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>31-Jul-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross incl. gold (IMF International Liquidity)</t>
+          <t>gross incl. gold</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>57.35</v>
+        <v>17.224</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1033,22 +1033,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>May-26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Central Bank of Egypt</t>
+          <t>IMF reserve template</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>07-Oct-26</t>
+          <t>31-May-26</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CBE-reported net international reserves; definition unverified and exceeds IMF gross, not comparable</t>
+          <t>reserves net of one-year drains (IMF reserve template); CBE reports a different net international reserves figure of 57.35 at Sep-26 that is not reconciled</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Central Bank of Egypt (over 7.5 months)</t>
+          <t>CBE (reported as over 7.5 months)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1271,11 +1271,6 @@
           <t>Stable</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Oct-26</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1307,7 +1302,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1317,7 +1312,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1329,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>31-Jul-26 (Seventh Review completed, $1.8B)</t>
+          <t>Seventh Review completed 31-Jul-26, $1.8B approved ($1.5B EFF, $272M RSF)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 (Eighth and final review; no primary source)</t>
+          <t>Eighth and final EFF review (with third RSF review), Q4-26, expected by mid-Dec-26; 15-Dec-26 Board date unconfirmed</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1368,40 +1363,50 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>FY25/26</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FY25/26E</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Q2-26</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1414,15 +1419,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
         <v>429.6</v>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>IMF WEO, 15-Oct-26</t>
         </is>
@@ -1435,15 +1442,17 @@
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" t="inlineStr">
         <is>
           <t>IMF WEO, 15-Oct-26</t>
         </is>
@@ -1462,7 +1471,9 @@
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1471,17 +1482,19 @@
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n">
         <v>-4.2</v>
       </c>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>IMF WEO, 15-Oct-26</t>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>IMF WEO via repo record, 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1492,15 +1505,17 @@
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
         <v>-12.1</v>
       </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>IMF WEO, 15-Oct-26</t>
         </is>
@@ -1512,26 +1527,30 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n">
         <v>3.5</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="D7" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n">
         <v>3.5</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="I7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Ministry of Finance of Egypt, FY24/25 outturn (fiscal year to Jun-25), Sep-26</t>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Moody's and S&amp;P via press, 16-Oct-26; fiscal years ending Jun (2025 = FY24/25, 2026 = FY25/26)</t>
         </is>
       </c>
     </row>
@@ -1541,22 +1560,28 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n">
+      <c r="B8" s="2" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>79.7</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>96.40000000000001</v>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n">
         <v>79.7</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Ministry of Finance / IIF, Jun-26 (budget-sector perimeter)</t>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Moody's via Daba Finance, 16-Oct-26; 2026 = Jun-26</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1598,9 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1588,7 +1615,9 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1603,7 +1632,9 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1613,12 +1644,20 @@
       </c>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
+      <c r="D12" s="2" t="n">
+        <v>59</v>
+      </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Moody's via Daba Finance, 16-Oct-26; 2026 = FY25/26</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>